<commit_message>
revised 1-5 handout and key
</commit_message>
<xml_diff>
--- a/handouts/chapter_1_5_handout.xlsx
+++ b/handouts/chapter_1_5_handout.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78AF1776-9407-41A2-919F-FADCE73D2F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{CB73943A-C465-40BE-817C-B9991112161C}"/>
+    <workbookView xWindow="3380" yWindow="3380" windowWidth="19200" windowHeight="11170" xr2:uid="{CB73943A-C465-40BE-817C-B9991112161C}"/>
   </bookViews>
   <sheets>
     <sheet name="Workbook" sheetId="2" r:id="rId1"/>
@@ -6582,6 +6582,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010070F75838E79B0E48B83E8E3F5479A3A2" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2b0c304636f8f537543cd13f583db9d4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xmlns:ns4="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f089f22c5ce4e61126931f7622145b2" ns3:_="" ns4:_="">
     <xsd:import namespace="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
@@ -6776,38 +6793,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBDDC771-C014-4A48-9FCA-802C556EA1D0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
-    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6830,9 +6819,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBDDC771-C014-4A48-9FCA-802C556EA1D0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
+    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>